<commit_message>
Add expected answers for Provisions and Calculator tabs; correct CPC s.28 page finding
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QyhGq4TAyzcfKLm3kLd6nF
</commit_message>
<xml_diff>
--- a/malaysia-police-powers-citizen-rights/review/praxis-rights-review-2026-10-13_QA-annotated.xlsx
+++ b/malaysia-police-powers-citizen-rights/review/praxis-rights-review-2026-10-13_QA-annotated.xlsx
@@ -642,13 +642,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" t="n">
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -27156,12 +27156,12 @@
       </c>
       <c r="M15" s="1" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NOT OK</t>
         </is>
       </c>
       <c r="N15" s="1" t="inlineStr">
         <is>
-          <t>Text and page reference consistent with the supplied reprint.</t>
+          <t>Approved as 'verified against ... p.39'. Section 28 begins on printed page 41 of the 2022 reprint (p.39 holds s.24). Transcription is accurate; the page check was not done.</t>
         </is>
       </c>
     </row>

</xml_diff>